<commit_message>
Update sample Excel file
</commit_message>
<xml_diff>
--- a/static/VRP_sample.xlsx
+++ b/static/VRP_sample.xlsx
@@ -2,15 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrapp\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6EB4FDB-6A43-4A6F-924A-5F088506EE9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDADC04-D278-4A6D-A053-1435A81BC947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="locations" sheetId="1" r:id="rId1"/>
@@ -23,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="46">
   <si>
     <t>lat</t>
   </si>
@@ -140,9 +135,6 @@
   </si>
   <si>
     <t>StartFromLastSolution</t>
-  </si>
-  <si>
-    <t>true</t>
   </si>
   <si>
     <t>True to use previous solution routes as a starting point and false to start from scratch</t>
@@ -3505,6 +3497,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3675,6 +3668,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3685,7 +3679,7 @@
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="3" max="3" width="131" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -3802,15 +3796,16 @@
       <c r="A11" t="s">
         <v>38</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" t="b">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
         <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3830,22 +3825,22 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>46</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>0</v>
@@ -3856,5 +3851,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>